<commit_message>
update bill of materials
</commit_message>
<xml_diff>
--- a/bom.xlsx
+++ b/bom.xlsx
@@ -1,15 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre.maia\Documents\GitHub\Optogenetics-Chamber\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08733A1E-95D4-4C80-8A2D-4371897B0E3F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -18,12 +24,142 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
+  <si>
+    <t>qty</t>
+  </si>
+  <si>
+    <t>item</t>
+  </si>
+  <si>
+    <t>detail</t>
+  </si>
+  <si>
+    <t>total cost</t>
+  </si>
+  <si>
+    <t>arduino mega headers</t>
+  </si>
+  <si>
+    <t>to stack shield on top of arduino</t>
+  </si>
+  <si>
+    <t>arduino mega</t>
+  </si>
+  <si>
+    <t>RGB LED</t>
+  </si>
+  <si>
+    <t>5mm common cathode</t>
+  </si>
+  <si>
+    <t>220 ohm resistor</t>
+  </si>
+  <si>
+    <t>flat cable</t>
+  </si>
+  <si>
+    <t>26awg 5mt</t>
+  </si>
+  <si>
+    <t>cost</t>
+  </si>
+  <si>
+    <t>unit cost (R$)</t>
+  </si>
+  <si>
+    <t>THT 1/4w kit 100 units</t>
+  </si>
+  <si>
+    <t>red led</t>
+  </si>
+  <si>
+    <t>5 mm for indication</t>
+  </si>
+  <si>
+    <t>mechanical switch</t>
+  </si>
+  <si>
+    <t>2 positions</t>
+  </si>
+  <si>
+    <t>power supply</t>
+  </si>
+  <si>
+    <t>12v 3a barrel connector</t>
+  </si>
+  <si>
+    <t>PLA filament</t>
+  </si>
+  <si>
+    <t>1kg</t>
+  </si>
+  <si>
+    <t>take advantage of all digital outputs</t>
+  </si>
+  <si>
+    <t>idc board connector</t>
+  </si>
+  <si>
+    <t>idc cable connector</t>
+  </si>
+  <si>
+    <t xml:space="preserve">THT </t>
+  </si>
+  <si>
+    <t>Users will need and IDC crimper to make cables</t>
+  </si>
+  <si>
+    <t>link</t>
+  </si>
+  <si>
+    <t>https://www.mercadolivre.com.br/shield-stacking-header-set-compatible-with-arduino-mega-2560/p/MLB2038789899?pdp_filters=item_id%3AMLB6641186364&amp;sid=bookmarks#polycard_client=wishlist&amp;wid=MLB6641186364&amp;sid=bookmarks</t>
+  </si>
+  <si>
+    <t>https://www.mercadolivre.com.br/filamento-pla-velvet-preto-1kg/p/MLB24741975?pdp_filters=item_id%3AMLB4411270263&amp;sid=bookmarks#polycard_client=wishlist&amp;wid=MLB4411270263&amp;sid=bookmarks</t>
+  </si>
+  <si>
+    <t>https://www.mercadolivre.com.br/fonte-alimentaco-12v-3a-pfita-led-cob-240l-cmera-bivolt/p/MLB2093977214?pdp_filters=item_id%3AMLB3966026211&amp;sid=bookmarks#polycard_client=wishlist&amp;wid=MLB3966026211&amp;sid=bookmarks</t>
+  </si>
+  <si>
+    <t>https://www.mercadolivre.com.br/20-pecas-micro-chave-interruptor-switch-pcb-2-posicao/up/MLBU596433095?pdp_filters=item_id%3AMLB1368421009&amp;sid=bookmarks#polycard_client=wishlist&amp;wid=MLB1368421009&amp;sid=bookmarks</t>
+  </si>
+  <si>
+    <t>https://www.mercadolivre.com.br/kit-led-5mm-difuso-10-vermelho/p/MLB39027228?pdp_filters=item_id%3AMLB4313543229&amp;sid=bookmarks#polycard_client=wishlist&amp;wid=MLB4313543229&amp;sid=bookmarks</t>
+  </si>
+  <si>
+    <t>https://www.mercadolivre.com.br/cabo-flat-cable-6-vias-26awg-colorido-lance-5mts/p/MLB2076010736?pdp_filters=item_id%3AMLB2018146342&amp;sid=bookmarks#polycard_client=wishlist&amp;wid=MLB2018146342&amp;sid=bookmarks</t>
+  </si>
+  <si>
+    <t>https://www.mercadolivre.com.br/kit-100un-resistor-220r-220-ohm-14w-5-carbono-cr25/up/MLBU3943781257?pdp_filters=item_id%3AMLB6735459884&amp;sid=bookmarks#polycard_client=wishlist&amp;wid=MLB6735459884&amp;sid=bookmarks</t>
+  </si>
+  <si>
+    <t>https://www.mercadolivre.com.br/10-pecas-led-5mm-alto-brilho-rgb-catodo-comum/up/MLBU1437892895?pdp_filters=item_id%3AMLB3294848783&amp;sid=bookmarks#polycard_client=wishlist&amp;wid=MLB3294848783&amp;sid=bookmarks</t>
+  </si>
+  <si>
+    <t>https://www.mercadolivre.com.br/placa-compativel-arduino-mega-2560-ch340-atmega2560--cabo/up/MLBU759484633?pdp_filters=item_id%3AMLB3367856807&amp;sid=bookmarks#polycard_client=wishlist&amp;wid=MLB3367856807&amp;sid=bookmarks</t>
+  </si>
+  <si>
+    <t>https://www.mercadolivre.com.br/10x--conector-barra-de-pinos-ds101310ssib1b-254mm-2x5/up/MLBU1749252615?pdp_filters=item_id%3AMLB3474477491&amp;sid=bookmarks#polycard_client=wishlist&amp;wid=MLB3474477491&amp;sid=bookmarks</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -46,13 +182,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -330,10 +469,275 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="43.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="3.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>55</v>
+      </c>
+      <c r="E2">
+        <f>C2*D2</f>
+        <v>55</v>
+      </c>
+      <c r="F2">
+        <f>SUM(E:E)</f>
+        <v>579</v>
+      </c>
+      <c r="G2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>135</v>
+      </c>
+      <c r="E3">
+        <f t="shared" ref="E3:E13" si="0">C3*D3</f>
+        <v>135</v>
+      </c>
+      <c r="G3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4">
+        <v>10</v>
+      </c>
+      <c r="D4">
+        <v>2</v>
+      </c>
+      <c r="E4">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="G4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5">
+        <v>10</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
+      </c>
+      <c r="E5">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="G5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>25</v>
+      </c>
+      <c r="E6">
+        <f>C6*D6</f>
+        <v>25</v>
+      </c>
+      <c r="G6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>35</v>
+      </c>
+      <c r="E7">
+        <f>C7*D7</f>
+        <v>35</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8">
+        <v>20</v>
+      </c>
+      <c r="D8">
+        <v>1.5</v>
+      </c>
+      <c r="E8">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+      <c r="G8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>19</v>
+      </c>
+      <c r="E9">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10">
+        <v>130</v>
+      </c>
+      <c r="E10">
+        <f t="shared" si="0"/>
+        <v>130</v>
+      </c>
+      <c r="G10" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11">
+        <v>10</v>
+      </c>
+      <c r="D11">
+        <v>5</v>
+      </c>
+      <c r="E11">
+        <f t="shared" si="0"/>
+        <v>50</v>
+      </c>
+      <c r="G11" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12">
+        <v>20</v>
+      </c>
+      <c r="D12">
+        <v>3</v>
+      </c>
+      <c r="E12">
+        <f t="shared" si="0"/>
+        <v>60</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="G9" r:id="rId1" location="polycard_client=wishlist&amp;wid=MLB3966026211&amp;sid=bookmarks" xr:uid="{154BE19C-F4A7-4E20-86AF-5951EDE15EBE}"/>
+    <hyperlink ref="G7" r:id="rId2" location="polycard_client=wishlist&amp;wid=MLB2018146342&amp;sid=bookmarks" xr:uid="{7714BB44-964F-452B-BE06-57BA2BBD25F5}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add cost for the mega board PCB shield
</commit_message>
<xml_diff>
--- a/bom.xlsx
+++ b/bom.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre.maia\Documents\GitHub\Optogenetics-Chamber\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08733A1E-95D4-4C80-8A2D-4371897B0E3F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F4A0007-23B6-42BF-8D16-12A3195D00BD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t>qty</t>
   </si>
@@ -142,6 +142,15 @@
   </si>
   <si>
     <t>https://www.mercadolivre.com.br/10x--conector-barra-de-pinos-ds101310ssib1b-254mm-2x5/up/MLBU1749252615?pdp_filters=item_id%3AMLB3474477491&amp;sid=bookmarks#polycard_client=wishlist&amp;wid=MLB3474477491&amp;sid=bookmarks</t>
+  </si>
+  <si>
+    <t>Custom printed circuit board</t>
+  </si>
+  <si>
+    <t>a shield for the mega board</t>
+  </si>
+  <si>
+    <t>jlcpcb.com</t>
   </si>
 </sst>
 </file>
@@ -470,10 +479,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="43.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="3.85546875" bestFit="1" customWidth="1"/>
   </cols>
@@ -520,7 +529,7 @@
       </c>
       <c r="F2">
         <f>SUM(E:E)</f>
-        <v>579</v>
+        <v>629</v>
       </c>
       <c r="G2" t="s">
         <v>29</v>
@@ -731,6 +740,27 @@
       <c r="E12">
         <f t="shared" si="0"/>
         <v>60</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>39</v>
+      </c>
+      <c r="B13" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13">
+        <v>1</v>
+      </c>
+      <c r="D13">
+        <v>50</v>
+      </c>
+      <c r="E13">
+        <f t="shared" si="0"/>
+        <v>50</v>
+      </c>
+      <c r="G13" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update bom and finish first version of PCBs
</commit_message>
<xml_diff>
--- a/bom.xlsx
+++ b/bom.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre.maia\Documents\GitHub\Optogenetics-Chamber\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F4A0007-23B6-42BF-8D16-12A3195D00BD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B5FE856-2C5B-44C6-B3B0-545D80672948}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="43">
   <si>
     <t>qty</t>
   </si>
@@ -63,9 +63,6 @@
     <t>26awg 5mt</t>
   </si>
   <si>
-    <t>cost</t>
-  </si>
-  <si>
     <t>unit cost (R$)</t>
   </si>
   <si>
@@ -151,13 +148,19 @@
   </si>
   <si>
     <t>jlcpcb.com</t>
+  </si>
+  <si>
+    <t>smaller pcb for holding LEDs</t>
+  </si>
+  <si>
+    <t>cost (BRL)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -169,6 +172,14 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -195,9 +206,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
@@ -479,7 +491,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.7109375" bestFit="1" customWidth="1"/>
@@ -498,16 +510,16 @@
         <v>0</v>
       </c>
       <c r="D1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E1" t="s">
-        <v>12</v>
+        <v>42</v>
       </c>
       <c r="F1" t="s">
         <v>3</v>
       </c>
       <c r="G1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -529,10 +541,10 @@
       </c>
       <c r="F2">
         <f>SUM(E:E)</f>
-        <v>629</v>
+        <v>829</v>
       </c>
       <c r="G2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -540,7 +552,7 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -549,11 +561,11 @@
         <v>135</v>
       </c>
       <c r="E3">
-        <f t="shared" ref="E3:E13" si="0">C3*D3</f>
+        <f t="shared" ref="E3:E14" si="0">C3*D3</f>
         <v>135</v>
       </c>
       <c r="G3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -574,15 +586,15 @@
         <v>20</v>
       </c>
       <c r="G4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" t="s">
         <v>15</v>
-      </c>
-      <c r="B5" t="s">
-        <v>16</v>
       </c>
       <c r="C5">
         <v>10</v>
@@ -595,7 +607,7 @@
         <v>20</v>
       </c>
       <c r="G5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -603,7 +615,7 @@
         <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C6">
         <v>1</v>
@@ -616,7 +628,7 @@
         <v>25</v>
       </c>
       <c r="G6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -637,15 +649,15 @@
         <v>35</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" t="s">
         <v>17</v>
-      </c>
-      <c r="B8" t="s">
-        <v>18</v>
       </c>
       <c r="C8">
         <v>20</v>
@@ -658,15 +670,15 @@
         <v>30</v>
       </c>
       <c r="G8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" t="s">
         <v>19</v>
-      </c>
-      <c r="B9" t="s">
-        <v>20</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -679,15 +691,15 @@
         <v>19</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" t="s">
         <v>21</v>
-      </c>
-      <c r="B10" t="s">
-        <v>22</v>
       </c>
       <c r="C10">
         <v>1</v>
@@ -700,15 +712,15 @@
         <v>130</v>
       </c>
       <c r="G10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C11">
         <v>10</v>
@@ -721,15 +733,15 @@
         <v>50</v>
       </c>
       <c r="G11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C12">
         <v>20</v>
@@ -744,10 +756,10 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>38</v>
+      </c>
+      <c r="B13" t="s">
         <v>39</v>
-      </c>
-      <c r="B13" t="s">
-        <v>40</v>
       </c>
       <c r="C13">
         <v>1</v>
@@ -760,7 +772,28 @@
         <v>50</v>
       </c>
       <c r="G13" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" t="s">
         <v>41</v>
+      </c>
+      <c r="C14">
+        <v>10</v>
+      </c>
+      <c r="D14">
+        <v>20</v>
+      </c>
+      <c r="E14">
+        <f t="shared" si="0"/>
+        <v>200</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -769,5 +802,6 @@
     <hyperlink ref="G7" r:id="rId2" location="polycard_client=wishlist&amp;wid=MLB2018146342&amp;sid=bookmarks" xr:uid="{7714BB44-964F-452B-BE06-57BA2BBD25F5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>